<commit_message>
Actualizando las responsabilidades del Objeto de dominio Residente
</commit_message>
<xml_diff>
--- a/Doo-Doc/Nueva Version Victus/Event Storming/ConjuntosResidenciales - Event Storming.xlsx
+++ b/Doo-Doc/Nueva Version Victus/Event Storming/ConjuntosResidenciales - Event Storming.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andre\Documents\DOO 2024 BD\DOO\victus-doc\Doo-Doc\Nueva Version Victus\Event Storming\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35F016F6-83A1-46EA-B2DF-1A13B637D482}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D7168F6-D241-4EF5-8163-9D569E75DEC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{36012E7C-B3F4-482B-AC16-7CCB81B9AE88}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="6" xr2:uid="{36012E7C-B3F4-482B-AC16-7CCB81B9AE88}"/>
   </bookViews>
   <sheets>
     <sheet name="Flujo de eventos en el tiempo" sheetId="61" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="425" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="204">
   <si>
     <t>Descripción</t>
   </si>
@@ -593,9 +593,6 @@
     <t>ZonInm-Pol0004</t>
   </si>
   <si>
-    <t>No es posible tener mas de un tipo inmueble que tenga el mismo número de vivienda más la misma zona inmueble.</t>
-  </si>
-  <si>
     <t>Se debe asegurar exista una zona inmueble.</t>
   </si>
   <si>
@@ -630,6 +627,36 @@
   </si>
   <si>
     <t>ConRes-Pol0005</t>
+  </si>
+  <si>
+    <t>La combinación de TipoInmueble, numeroVivienda y ZonaInmueble debe ser única.</t>
+  </si>
+  <si>
+    <t>TipoInmueble y ZonaInmueble deben ser referencias válidas.</t>
+  </si>
+  <si>
+    <t>Sistema</t>
+  </si>
+  <si>
+    <t>Asegurar que el identificador del inmueble que se decea buscar exista.</t>
+  </si>
+  <si>
+    <t>Inmueble-Pol0005</t>
+  </si>
+  <si>
+    <t>Inmueble-Pol0006</t>
+  </si>
+  <si>
+    <t>Si se cambia TipoInmueble, numeroVivienda o ZonaInmueble, la combinación debe seguir siendo única.</t>
+  </si>
+  <si>
+    <t>Inmueble-Pol0007</t>
+  </si>
+  <si>
+    <t>Inmueble-Pol0008</t>
+  </si>
+  <si>
+    <t>El Inmueble no debe estar asignado a ningún residente antes de ser eliminado.</t>
   </si>
 </sst>
 </file>
@@ -695,7 +722,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="19">
+  <fills count="22">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -804,8 +831,26 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="26">
+  <borders count="27">
     <border>
       <left/>
       <right/>
@@ -1132,12 +1177,27 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thick">
+        <color indexed="64"/>
+      </left>
+      <right style="thick">
+        <color indexed="64"/>
+      </right>
+      <top style="thick">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thick">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="111">
+  <cellXfs count="143">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1263,6 +1323,9 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1272,15 +1335,42 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1308,41 +1398,119 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1350,114 +1518,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="13" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="13" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="13" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1465,6 +1525,102 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2017,83 +2173,83 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="57" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
-      <c r="G1" s="46"/>
-      <c r="H1" s="46"/>
-      <c r="I1" s="46"/>
-      <c r="J1" s="46"/>
-      <c r="K1" s="46"/>
-      <c r="L1" s="46"/>
-      <c r="M1" s="46"/>
-      <c r="N1" s="46"/>
+      <c r="B1" s="57"/>
+      <c r="C1" s="57"/>
+      <c r="D1" s="57"/>
+      <c r="E1" s="57"/>
+      <c r="F1" s="57"/>
+      <c r="G1" s="57"/>
+      <c r="H1" s="57"/>
+      <c r="I1" s="57"/>
+      <c r="J1" s="57"/>
+      <c r="K1" s="57"/>
+      <c r="L1" s="57"/>
+      <c r="M1" s="57"/>
+      <c r="N1" s="57"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="56" t="s">
+      <c r="B2" s="66" t="s">
         <v>29</v>
       </c>
-      <c r="C2" s="56"/>
-      <c r="D2" s="56"/>
-      <c r="E2" s="56"/>
-      <c r="F2" s="56"/>
-      <c r="G2" s="56"/>
-      <c r="H2" s="56"/>
-      <c r="I2" s="56"/>
-      <c r="J2" s="56"/>
-      <c r="K2" s="56"/>
-      <c r="L2" s="56"/>
-      <c r="M2" s="57"/>
+      <c r="C2" s="66"/>
+      <c r="D2" s="66"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="66"/>
+      <c r="G2" s="66"/>
+      <c r="H2" s="66"/>
+      <c r="I2" s="66"/>
+      <c r="J2" s="66"/>
+      <c r="K2" s="66"/>
+      <c r="L2" s="66"/>
+      <c r="M2" s="67"/>
       <c r="N2" s="3"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="64" t="str">
+      <c r="B3" s="68" t="str">
         <f>'Listado Objetos de Dominio'!B4</f>
         <v>Objeto de dominio que representa cada una de las comunidades habitacionales organizadas en un sistema. Abarca la totalidad de los elementos que componen el conjunto, desde las unidades habitacionales individuales (inmuebles) hasta las zonas comunes.</v>
       </c>
-      <c r="C3" s="64"/>
-      <c r="D3" s="64"/>
-      <c r="E3" s="64"/>
-      <c r="F3" s="64"/>
-      <c r="G3" s="64"/>
-      <c r="H3" s="64"/>
-      <c r="I3" s="64"/>
-      <c r="J3" s="64"/>
-      <c r="K3" s="64"/>
-      <c r="L3" s="64"/>
-      <c r="M3" s="65"/>
+      <c r="C3" s="68"/>
+      <c r="D3" s="68"/>
+      <c r="E3" s="68"/>
+      <c r="F3" s="68"/>
+      <c r="G3" s="68"/>
+      <c r="H3" s="68"/>
+      <c r="I3" s="68"/>
+      <c r="J3" s="68"/>
+      <c r="K3" s="68"/>
+      <c r="L3" s="68"/>
+      <c r="M3" s="69"/>
       <c r="N3" s="4"/>
     </row>
     <row r="4" spans="1:14" ht="29.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="48" t="s">
+      <c r="B4" s="53" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="48"/>
+      <c r="C4" s="53"/>
       <c r="D4" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="E4" s="66" t="s">
+      <c r="E4" s="54" t="s">
         <v>19</v>
       </c>
-      <c r="F4" s="66"/>
-      <c r="G4" s="51" t="s">
+      <c r="F4" s="54"/>
+      <c r="G4" s="61" t="s">
         <v>13</v>
       </c>
-      <c r="H4" s="51"/>
+      <c r="H4" s="61"/>
       <c r="I4" s="9" t="s">
         <v>14</v>
       </c>
@@ -2103,52 +2259,52 @@
       <c r="K4" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="L4" s="54" t="s">
+      <c r="L4" s="64" t="s">
         <v>17</v>
       </c>
-      <c r="M4" s="55" t="s">
+      <c r="M4" s="65" t="s">
         <v>18</v>
       </c>
       <c r="N4" s="4"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A5" s="47" t="s">
+      <c r="A5" s="58" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="48" t="s">
+      <c r="B5" s="53" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="48" t="s">
+      <c r="C5" s="53" t="s">
         <v>0</v>
       </c>
-      <c r="D5" s="67" t="s">
+      <c r="D5" s="55" t="s">
         <v>23</v>
       </c>
-      <c r="E5" s="66" t="s">
+      <c r="E5" s="54" t="s">
         <v>20</v>
       </c>
-      <c r="F5" s="66"/>
-      <c r="G5" s="49" t="s">
+      <c r="F5" s="54"/>
+      <c r="G5" s="59" t="s">
         <v>7</v>
       </c>
-      <c r="H5" s="49"/>
-      <c r="I5" s="52" t="s">
+      <c r="H5" s="59"/>
+      <c r="I5" s="62" t="s">
         <v>15</v>
       </c>
-      <c r="J5" s="53" t="s">
+      <c r="J5" s="63" t="s">
         <v>8</v>
       </c>
-      <c r="K5" s="50" t="s">
+      <c r="K5" s="60" t="s">
         <v>10</v>
       </c>
-      <c r="L5" s="54"/>
-      <c r="M5" s="55"/>
+      <c r="L5" s="64"/>
+      <c r="M5" s="65"/>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A6" s="47"/>
-      <c r="B6" s="48"/>
-      <c r="C6" s="48"/>
-      <c r="D6" s="68"/>
+      <c r="A6" s="58"/>
+      <c r="B6" s="53"/>
+      <c r="C6" s="53"/>
+      <c r="D6" s="56"/>
       <c r="E6" s="11" t="s">
         <v>21</v>
       </c>
@@ -2161,39 +2317,39 @@
       <c r="H6" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="I6" s="52"/>
-      <c r="J6" s="53"/>
-      <c r="K6" s="50"/>
-      <c r="L6" s="54"/>
-      <c r="M6" s="55"/>
+      <c r="I6" s="62"/>
+      <c r="J6" s="63"/>
+      <c r="K6" s="60"/>
+      <c r="L6" s="64"/>
+      <c r="M6" s="65"/>
     </row>
     <row r="7" spans="1:14" ht="87.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="61" t="s">
+      <c r="A7" s="50" t="s">
         <v>45</v>
       </c>
-      <c r="B7" s="58" t="s">
+      <c r="B7" s="47" t="s">
         <v>46</v>
       </c>
-      <c r="C7" s="58" t="s">
+      <c r="C7" s="47" t="s">
         <v>47</v>
       </c>
-      <c r="D7" s="58" t="s">
+      <c r="D7" s="47" t="s">
         <v>29</v>
       </c>
-      <c r="E7" s="58"/>
-      <c r="F7" s="58"/>
-      <c r="G7" s="43" t="s">
+      <c r="E7" s="47"/>
+      <c r="F7" s="47"/>
+      <c r="G7" s="44" t="s">
         <v>48</v>
       </c>
-      <c r="H7" s="43" t="s">
+      <c r="H7" s="44" t="s">
         <v>158</v>
       </c>
-      <c r="I7" s="58"/>
-      <c r="J7" s="58" t="s">
+      <c r="I7" s="47"/>
+      <c r="J7" s="47" t="s">
         <v>44</v>
       </c>
-      <c r="K7" s="58"/>
-      <c r="L7" s="58" t="s">
+      <c r="K7" s="47"/>
+      <c r="L7" s="47" t="s">
         <v>36</v>
       </c>
       <c r="M7" s="26" t="s">
@@ -2201,104 +2357,104 @@
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A8" s="62"/>
-      <c r="B8" s="59"/>
-      <c r="C8" s="59"/>
-      <c r="D8" s="59"/>
-      <c r="E8" s="59"/>
-      <c r="F8" s="59"/>
-      <c r="G8" s="44"/>
-      <c r="H8" s="44"/>
-      <c r="I8" s="59"/>
-      <c r="J8" s="59"/>
-      <c r="K8" s="59"/>
-      <c r="L8" s="59"/>
+      <c r="A8" s="51"/>
+      <c r="B8" s="48"/>
+      <c r="C8" s="48"/>
+      <c r="D8" s="48"/>
+      <c r="E8" s="48"/>
+      <c r="F8" s="48"/>
+      <c r="G8" s="45"/>
+      <c r="H8" s="45"/>
+      <c r="I8" s="48"/>
+      <c r="J8" s="48"/>
+      <c r="K8" s="48"/>
+      <c r="L8" s="48"/>
       <c r="M8" s="26" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A9" s="62"/>
-      <c r="B9" s="59"/>
-      <c r="C9" s="59"/>
-      <c r="D9" s="59"/>
-      <c r="E9" s="59"/>
-      <c r="F9" s="59"/>
-      <c r="G9" s="45"/>
-      <c r="H9" s="45"/>
-      <c r="I9" s="59"/>
-      <c r="J9" s="59"/>
-      <c r="K9" s="59"/>
-      <c r="L9" s="59"/>
+      <c r="A9" s="51"/>
+      <c r="B9" s="48"/>
+      <c r="C9" s="48"/>
+      <c r="D9" s="48"/>
+      <c r="E9" s="48"/>
+      <c r="F9" s="48"/>
+      <c r="G9" s="46"/>
+      <c r="H9" s="46"/>
+      <c r="I9" s="48"/>
+      <c r="J9" s="48"/>
+      <c r="K9" s="48"/>
+      <c r="L9" s="48"/>
       <c r="M9" s="26" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="57.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="62"/>
-      <c r="B10" s="59"/>
-      <c r="C10" s="59"/>
-      <c r="D10" s="59"/>
-      <c r="E10" s="59"/>
-      <c r="F10" s="59"/>
-      <c r="G10" s="69" t="s">
+      <c r="A10" s="51"/>
+      <c r="B10" s="48"/>
+      <c r="C10" s="48"/>
+      <c r="D10" s="48"/>
+      <c r="E10" s="48"/>
+      <c r="F10" s="48"/>
+      <c r="G10" s="43" t="s">
         <v>51</v>
       </c>
-      <c r="H10" s="69" t="s">
+      <c r="H10" s="43" t="s">
         <v>160</v>
       </c>
-      <c r="I10" s="59"/>
-      <c r="J10" s="59"/>
-      <c r="K10" s="59"/>
-      <c r="L10" s="59"/>
+      <c r="I10" s="48"/>
+      <c r="J10" s="48"/>
+      <c r="K10" s="48"/>
+      <c r="L10" s="48"/>
       <c r="M10" s="26" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="11" spans="1:14" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="63"/>
-      <c r="B11" s="60"/>
-      <c r="C11" s="60"/>
-      <c r="D11" s="60"/>
-      <c r="E11" s="60"/>
-      <c r="F11" s="60"/>
-      <c r="G11" s="69"/>
-      <c r="H11" s="69"/>
-      <c r="I11" s="60"/>
-      <c r="J11" s="60"/>
-      <c r="K11" s="60"/>
-      <c r="L11" s="60"/>
+      <c r="A11" s="52"/>
+      <c r="B11" s="49"/>
+      <c r="C11" s="49"/>
+      <c r="D11" s="49"/>
+      <c r="E11" s="49"/>
+      <c r="F11" s="49"/>
+      <c r="G11" s="43"/>
+      <c r="H11" s="43"/>
+      <c r="I11" s="49"/>
+      <c r="J11" s="49"/>
+      <c r="K11" s="49"/>
+      <c r="L11" s="49"/>
       <c r="M11" s="26" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="12" spans="1:14" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="61" t="s">
+      <c r="A12" s="50" t="s">
         <v>45</v>
       </c>
-      <c r="B12" s="58" t="s">
+      <c r="B12" s="47" t="s">
         <v>49</v>
       </c>
-      <c r="C12" s="58" t="s">
+      <c r="C12" s="47" t="s">
         <v>50</v>
       </c>
-      <c r="D12" s="58" t="s">
+      <c r="D12" s="47" t="s">
         <v>29</v>
       </c>
-      <c r="E12" s="58"/>
-      <c r="F12" s="58"/>
-      <c r="G12" s="43" t="s">
+      <c r="E12" s="47"/>
+      <c r="F12" s="47"/>
+      <c r="G12" s="44" t="s">
         <v>56</v>
       </c>
-      <c r="H12" s="43" t="s">
+      <c r="H12" s="44" t="s">
         <v>54</v>
       </c>
-      <c r="I12" s="58"/>
-      <c r="J12" s="58" t="s">
+      <c r="I12" s="47"/>
+      <c r="J12" s="47" t="s">
         <v>32</v>
       </c>
-      <c r="K12" s="58"/>
-      <c r="L12" s="58" t="s">
+      <c r="K12" s="47"/>
+      <c r="L12" s="47" t="s">
         <v>44</v>
       </c>
       <c r="M12" s="26" t="s">
@@ -2306,52 +2462,52 @@
       </c>
     </row>
     <row r="13" spans="1:14" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="62"/>
-      <c r="B13" s="59"/>
-      <c r="C13" s="59"/>
-      <c r="D13" s="59"/>
-      <c r="E13" s="59"/>
-      <c r="F13" s="59"/>
-      <c r="G13" s="44"/>
-      <c r="H13" s="44"/>
-      <c r="I13" s="59"/>
-      <c r="J13" s="59"/>
-      <c r="K13" s="59"/>
-      <c r="L13" s="59"/>
+      <c r="A13" s="51"/>
+      <c r="B13" s="48"/>
+      <c r="C13" s="48"/>
+      <c r="D13" s="48"/>
+      <c r="E13" s="48"/>
+      <c r="F13" s="48"/>
+      <c r="G13" s="45"/>
+      <c r="H13" s="45"/>
+      <c r="I13" s="48"/>
+      <c r="J13" s="48"/>
+      <c r="K13" s="48"/>
+      <c r="L13" s="48"/>
       <c r="M13" s="26" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="14" spans="1:14" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="62"/>
-      <c r="B14" s="59"/>
-      <c r="C14" s="59"/>
-      <c r="D14" s="59"/>
-      <c r="E14" s="59"/>
-      <c r="F14" s="59"/>
-      <c r="G14" s="44"/>
-      <c r="H14" s="44"/>
-      <c r="I14" s="59"/>
-      <c r="J14" s="59"/>
-      <c r="K14" s="59"/>
-      <c r="L14" s="59"/>
+      <c r="A14" s="51"/>
+      <c r="B14" s="48"/>
+      <c r="C14" s="48"/>
+      <c r="D14" s="48"/>
+      <c r="E14" s="48"/>
+      <c r="F14" s="48"/>
+      <c r="G14" s="45"/>
+      <c r="H14" s="45"/>
+      <c r="I14" s="48"/>
+      <c r="J14" s="48"/>
+      <c r="K14" s="48"/>
+      <c r="L14" s="48"/>
       <c r="M14" s="26" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="15" spans="1:14" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="63"/>
-      <c r="B15" s="60"/>
-      <c r="C15" s="60"/>
-      <c r="D15" s="60"/>
-      <c r="E15" s="60"/>
-      <c r="F15" s="60"/>
-      <c r="G15" s="44"/>
-      <c r="H15" s="44"/>
-      <c r="I15" s="60"/>
-      <c r="J15" s="60"/>
-      <c r="K15" s="60"/>
-      <c r="L15" s="60"/>
+      <c r="A15" s="52"/>
+      <c r="B15" s="49"/>
+      <c r="C15" s="49"/>
+      <c r="D15" s="49"/>
+      <c r="E15" s="49"/>
+      <c r="F15" s="49"/>
+      <c r="G15" s="45"/>
+      <c r="H15" s="45"/>
+      <c r="I15" s="49"/>
+      <c r="J15" s="49"/>
+      <c r="K15" s="49"/>
+      <c r="L15" s="49"/>
       <c r="M15" s="26" t="s">
         <v>89</v>
       </c>
@@ -2361,21 +2517,21 @@
         <v>45</v>
       </c>
       <c r="B16" s="35" t="s">
+        <v>189</v>
+      </c>
+      <c r="C16" s="35" t="s">
         <v>190</v>
-      </c>
-      <c r="C16" s="35" t="s">
-        <v>191</v>
       </c>
       <c r="D16" s="35" t="s">
         <v>29</v>
       </c>
       <c r="E16" s="35"/>
       <c r="F16" s="35"/>
-      <c r="G16" s="45"/>
-      <c r="H16" s="45"/>
+      <c r="G16" s="46"/>
+      <c r="H16" s="46"/>
       <c r="I16" s="35"/>
       <c r="J16" s="35" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="K16" s="35"/>
       <c r="L16" s="35" t="s">
@@ -2400,10 +2556,10 @@
       </c>
       <c r="E17" s="22"/>
       <c r="F17" s="22"/>
-      <c r="G17" s="69" t="s">
-        <v>193</v>
-      </c>
-      <c r="H17" s="69" t="s">
+      <c r="G17" s="43" t="s">
+        <v>192</v>
+      </c>
+      <c r="H17" s="43" t="s">
         <v>160</v>
       </c>
       <c r="I17" s="22"/>
@@ -2433,8 +2589,8 @@
       </c>
       <c r="E18" s="22"/>
       <c r="F18" s="22"/>
-      <c r="G18" s="69"/>
-      <c r="H18" s="69"/>
+      <c r="G18" s="43"/>
+      <c r="H18" s="43"/>
       <c r="I18" s="22"/>
       <c r="J18" s="22" t="s">
         <v>34</v>
@@ -2462,10 +2618,10 @@
       </c>
       <c r="E19" s="22"/>
       <c r="F19" s="22"/>
-      <c r="G19" s="43" t="s">
-        <v>194</v>
-      </c>
-      <c r="H19" s="43" t="s">
+      <c r="G19" s="44" t="s">
+        <v>193</v>
+      </c>
+      <c r="H19" s="44" t="s">
         <v>159</v>
       </c>
       <c r="I19" s="22"/>
@@ -2495,8 +2651,8 @@
       </c>
       <c r="E20" s="22"/>
       <c r="F20" s="22"/>
-      <c r="G20" s="44"/>
-      <c r="H20" s="44"/>
+      <c r="G20" s="45"/>
+      <c r="H20" s="45"/>
       <c r="I20" s="22"/>
       <c r="J20" s="22" t="s">
         <v>41</v>
@@ -2524,8 +2680,8 @@
       </c>
       <c r="E21" s="22"/>
       <c r="F21" s="22"/>
-      <c r="G21" s="45"/>
-      <c r="H21" s="45"/>
+      <c r="G21" s="46"/>
+      <c r="H21" s="46"/>
       <c r="I21" s="22"/>
       <c r="J21" s="22" t="s">
         <v>36</v>
@@ -2540,37 +2696,6 @@
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="G10:G11"/>
-    <mergeCell ref="H10:H11"/>
-    <mergeCell ref="G12:G16"/>
-    <mergeCell ref="G17:G18"/>
-    <mergeCell ref="H17:H18"/>
-    <mergeCell ref="G19:G21"/>
-    <mergeCell ref="H19:H21"/>
-    <mergeCell ref="B12:B15"/>
-    <mergeCell ref="A12:A15"/>
-    <mergeCell ref="F12:F15"/>
-    <mergeCell ref="E12:E15"/>
-    <mergeCell ref="D12:D15"/>
-    <mergeCell ref="C12:C15"/>
-    <mergeCell ref="L12:L15"/>
-    <mergeCell ref="K12:K15"/>
-    <mergeCell ref="J12:J15"/>
-    <mergeCell ref="I12:I15"/>
-    <mergeCell ref="H12:H16"/>
-    <mergeCell ref="L7:L11"/>
-    <mergeCell ref="K7:K11"/>
-    <mergeCell ref="J7:J11"/>
-    <mergeCell ref="I7:I11"/>
-    <mergeCell ref="H7:H9"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="E4:F4"/>
-    <mergeCell ref="E5:F5"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="F7:F11"/>
-    <mergeCell ref="E7:E11"/>
-    <mergeCell ref="D7:D11"/>
-    <mergeCell ref="C7:C11"/>
     <mergeCell ref="G7:G9"/>
     <mergeCell ref="A1:N1"/>
     <mergeCell ref="A5:A6"/>
@@ -2587,6 +2712,37 @@
     <mergeCell ref="B7:B11"/>
     <mergeCell ref="A7:A11"/>
     <mergeCell ref="B3:M3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="F7:F11"/>
+    <mergeCell ref="E7:E11"/>
+    <mergeCell ref="D7:D11"/>
+    <mergeCell ref="C7:C11"/>
+    <mergeCell ref="L7:L11"/>
+    <mergeCell ref="K7:K11"/>
+    <mergeCell ref="J7:J11"/>
+    <mergeCell ref="I7:I11"/>
+    <mergeCell ref="H7:H9"/>
+    <mergeCell ref="L12:L15"/>
+    <mergeCell ref="K12:K15"/>
+    <mergeCell ref="J12:J15"/>
+    <mergeCell ref="I12:I15"/>
+    <mergeCell ref="H12:H16"/>
+    <mergeCell ref="G19:G21"/>
+    <mergeCell ref="H19:H21"/>
+    <mergeCell ref="B12:B15"/>
+    <mergeCell ref="A12:A15"/>
+    <mergeCell ref="F12:F15"/>
+    <mergeCell ref="E12:E15"/>
+    <mergeCell ref="D12:D15"/>
+    <mergeCell ref="C12:C15"/>
+    <mergeCell ref="G10:G11"/>
+    <mergeCell ref="H10:H11"/>
+    <mergeCell ref="G12:G16"/>
+    <mergeCell ref="G17:G18"/>
+    <mergeCell ref="H17:H18"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <hyperlinks>
@@ -2627,83 +2783,83 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="57" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
-      <c r="G1" s="46"/>
-      <c r="H1" s="46"/>
-      <c r="I1" s="46"/>
-      <c r="J1" s="46"/>
-      <c r="K1" s="46"/>
-      <c r="L1" s="46"/>
-      <c r="M1" s="46"/>
-      <c r="N1" s="46"/>
+      <c r="B1" s="57"/>
+      <c r="C1" s="57"/>
+      <c r="D1" s="57"/>
+      <c r="E1" s="57"/>
+      <c r="F1" s="57"/>
+      <c r="G1" s="57"/>
+      <c r="H1" s="57"/>
+      <c r="I1" s="57"/>
+      <c r="J1" s="57"/>
+      <c r="K1" s="57"/>
+      <c r="L1" s="57"/>
+      <c r="M1" s="57"/>
+      <c r="N1" s="57"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="72" t="s">
+      <c r="B2" s="78" t="s">
         <v>30</v>
       </c>
-      <c r="C2" s="73"/>
-      <c r="D2" s="73"/>
-      <c r="E2" s="73"/>
-      <c r="F2" s="73"/>
-      <c r="G2" s="73"/>
-      <c r="H2" s="73"/>
-      <c r="I2" s="73"/>
-      <c r="J2" s="73"/>
-      <c r="K2" s="73"/>
-      <c r="L2" s="73"/>
-      <c r="M2" s="74"/>
+      <c r="C2" s="79"/>
+      <c r="D2" s="79"/>
+      <c r="E2" s="79"/>
+      <c r="F2" s="79"/>
+      <c r="G2" s="79"/>
+      <c r="H2" s="79"/>
+      <c r="I2" s="79"/>
+      <c r="J2" s="79"/>
+      <c r="K2" s="79"/>
+      <c r="L2" s="79"/>
+      <c r="M2" s="80"/>
       <c r="N2" s="3"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="75" t="str">
+      <c r="B3" s="81" t="str">
         <f>'Listado Objetos de Dominio'!$B$5</f>
         <v>Objeto de dominio que representa a cada una de las zonas comunes que se encuentran dentro de un conjunto residencial para que los residentes puedan reservar esos espacios y porder usarlos.</v>
       </c>
-      <c r="C3" s="76"/>
-      <c r="D3" s="76"/>
-      <c r="E3" s="76"/>
-      <c r="F3" s="76"/>
-      <c r="G3" s="76"/>
-      <c r="H3" s="76"/>
-      <c r="I3" s="76"/>
-      <c r="J3" s="76"/>
-      <c r="K3" s="76"/>
-      <c r="L3" s="76"/>
-      <c r="M3" s="77"/>
+      <c r="C3" s="82"/>
+      <c r="D3" s="82"/>
+      <c r="E3" s="82"/>
+      <c r="F3" s="82"/>
+      <c r="G3" s="82"/>
+      <c r="H3" s="82"/>
+      <c r="I3" s="82"/>
+      <c r="J3" s="82"/>
+      <c r="K3" s="82"/>
+      <c r="L3" s="82"/>
+      <c r="M3" s="83"/>
       <c r="N3" s="4"/>
     </row>
     <row r="4" spans="1:14" ht="37.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="78" t="s">
+      <c r="B4" s="84" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="79"/>
+      <c r="C4" s="85"/>
       <c r="D4" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="E4" s="80" t="s">
+      <c r="E4" s="86" t="s">
         <v>19</v>
       </c>
-      <c r="F4" s="81"/>
-      <c r="G4" s="82" t="s">
+      <c r="F4" s="87"/>
+      <c r="G4" s="88" t="s">
         <v>13</v>
       </c>
-      <c r="H4" s="83"/>
+      <c r="H4" s="89"/>
       <c r="I4" s="9" t="s">
         <v>14</v>
       </c>
@@ -2713,52 +2869,52 @@
       <c r="K4" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="L4" s="84" t="s">
+      <c r="L4" s="90" t="s">
         <v>17</v>
       </c>
-      <c r="M4" s="87" t="s">
+      <c r="M4" s="93" t="s">
         <v>18</v>
       </c>
       <c r="N4" s="4"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A5" s="98" t="s">
+      <c r="A5" s="104" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="100" t="s">
+      <c r="B5" s="76" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="100" t="s">
+      <c r="C5" s="76" t="s">
         <v>0</v>
       </c>
-      <c r="D5" s="67" t="s">
+      <c r="D5" s="55" t="s">
         <v>23</v>
       </c>
-      <c r="E5" s="80" t="s">
+      <c r="E5" s="86" t="s">
         <v>20</v>
       </c>
-      <c r="F5" s="81"/>
-      <c r="G5" s="90" t="s">
+      <c r="F5" s="87"/>
+      <c r="G5" s="96" t="s">
         <v>7</v>
       </c>
-      <c r="H5" s="91"/>
-      <c r="I5" s="94" t="s">
+      <c r="H5" s="97"/>
+      <c r="I5" s="100" t="s">
         <v>15</v>
       </c>
-      <c r="J5" s="96" t="s">
+      <c r="J5" s="102" t="s">
         <v>8</v>
       </c>
-      <c r="K5" s="92" t="s">
+      <c r="K5" s="98" t="s">
         <v>10</v>
       </c>
-      <c r="L5" s="85"/>
-      <c r="M5" s="88"/>
+      <c r="L5" s="91"/>
+      <c r="M5" s="94"/>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A6" s="99"/>
-      <c r="B6" s="101"/>
-      <c r="C6" s="101"/>
-      <c r="D6" s="68"/>
+      <c r="A6" s="105"/>
+      <c r="B6" s="77"/>
+      <c r="C6" s="77"/>
+      <c r="D6" s="56"/>
       <c r="E6" s="11" t="s">
         <v>21</v>
       </c>
@@ -2771,29 +2927,29 @@
       <c r="H6" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="I6" s="95"/>
-      <c r="J6" s="97"/>
-      <c r="K6" s="93"/>
-      <c r="L6" s="86"/>
-      <c r="M6" s="89"/>
+      <c r="I6" s="101"/>
+      <c r="J6" s="103"/>
+      <c r="K6" s="99"/>
+      <c r="L6" s="92"/>
+      <c r="M6" s="95"/>
     </row>
     <row r="7" spans="1:14" ht="88.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="105" t="s">
+      <c r="A7" s="70" t="s">
         <v>31</v>
       </c>
-      <c r="B7" s="43" t="s">
+      <c r="B7" s="44" t="s">
         <v>161</v>
       </c>
-      <c r="C7" s="43" t="s">
+      <c r="C7" s="44" t="s">
         <v>64</v>
       </c>
-      <c r="D7" s="43" t="s">
+      <c r="D7" s="44" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="43" t="s">
+      <c r="E7" s="44" t="s">
         <v>63</v>
       </c>
-      <c r="F7" s="43" t="s">
+      <c r="F7" s="44" t="s">
         <v>62</v>
       </c>
       <c r="G7" s="22" t="s">
@@ -2802,12 +2958,12 @@
       <c r="H7" s="33" t="s">
         <v>162</v>
       </c>
-      <c r="I7" s="43"/>
-      <c r="J7" s="43" t="s">
+      <c r="I7" s="44"/>
+      <c r="J7" s="44" t="s">
         <v>37</v>
       </c>
-      <c r="K7" s="43"/>
-      <c r="L7" s="43" t="s">
+      <c r="K7" s="44"/>
+      <c r="L7" s="44" t="s">
         <v>38</v>
       </c>
       <c r="M7" s="24" t="s">
@@ -2815,54 +2971,54 @@
       </c>
     </row>
     <row r="8" spans="1:14" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="106"/>
-      <c r="B8" s="44"/>
-      <c r="C8" s="44"/>
-      <c r="D8" s="44"/>
-      <c r="E8" s="44"/>
-      <c r="F8" s="44"/>
-      <c r="G8" s="43" t="s">
+      <c r="A8" s="71"/>
+      <c r="B8" s="45"/>
+      <c r="C8" s="45"/>
+      <c r="D8" s="45"/>
+      <c r="E8" s="45"/>
+      <c r="F8" s="45"/>
+      <c r="G8" s="44" t="s">
         <v>71</v>
       </c>
-      <c r="H8" s="43" t="s">
+      <c r="H8" s="44" t="s">
         <v>163</v>
       </c>
-      <c r="I8" s="44"/>
-      <c r="J8" s="44"/>
-      <c r="K8" s="44"/>
-      <c r="L8" s="44"/>
-      <c r="M8" s="70" t="s">
+      <c r="I8" s="45"/>
+      <c r="J8" s="45"/>
+      <c r="K8" s="45"/>
+      <c r="L8" s="45"/>
+      <c r="M8" s="106" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="9" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="106"/>
-      <c r="B9" s="44"/>
-      <c r="C9" s="44"/>
-      <c r="D9" s="44"/>
-      <c r="E9" s="44"/>
-      <c r="F9" s="44"/>
-      <c r="G9" s="44"/>
-      <c r="H9" s="44"/>
-      <c r="I9" s="44"/>
-      <c r="J9" s="44"/>
-      <c r="K9" s="44"/>
-      <c r="L9" s="44"/>
-      <c r="M9" s="71"/>
+      <c r="A9" s="71"/>
+      <c r="B9" s="45"/>
+      <c r="C9" s="45"/>
+      <c r="D9" s="45"/>
+      <c r="E9" s="45"/>
+      <c r="F9" s="45"/>
+      <c r="G9" s="45"/>
+      <c r="H9" s="45"/>
+      <c r="I9" s="45"/>
+      <c r="J9" s="45"/>
+      <c r="K9" s="45"/>
+      <c r="L9" s="45"/>
+      <c r="M9" s="107"/>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A10" s="107"/>
-      <c r="B10" s="45"/>
-      <c r="C10" s="45"/>
-      <c r="D10" s="45"/>
-      <c r="E10" s="45"/>
-      <c r="F10" s="45"/>
-      <c r="G10" s="45"/>
-      <c r="H10" s="45"/>
-      <c r="I10" s="45"/>
-      <c r="J10" s="45"/>
-      <c r="K10" s="45"/>
-      <c r="L10" s="45"/>
+      <c r="A10" s="72"/>
+      <c r="B10" s="46"/>
+      <c r="C10" s="46"/>
+      <c r="D10" s="46"/>
+      <c r="E10" s="46"/>
+      <c r="F10" s="46"/>
+      <c r="G10" s="46"/>
+      <c r="H10" s="46"/>
+      <c r="I10" s="46"/>
+      <c r="J10" s="46"/>
+      <c r="K10" s="46"/>
+      <c r="L10" s="46"/>
       <c r="M10" s="31" t="s">
         <v>72</v>
       </c>
@@ -2871,33 +3027,33 @@
       <c r="A11" s="25" t="s">
         <v>43</v>
       </c>
-      <c r="B11" s="58" t="s">
+      <c r="B11" s="47" t="s">
         <v>67</v>
       </c>
-      <c r="C11" s="58" t="s">
+      <c r="C11" s="47" t="s">
         <v>68</v>
       </c>
-      <c r="D11" s="58" t="s">
+      <c r="D11" s="47" t="s">
         <v>30</v>
       </c>
-      <c r="E11" s="58" t="s">
+      <c r="E11" s="47" t="s">
         <v>63</v>
       </c>
-      <c r="F11" s="58" t="s">
+      <c r="F11" s="47" t="s">
         <v>70</v>
       </c>
-      <c r="G11" s="58" t="s">
+      <c r="G11" s="47" t="s">
         <v>164</v>
       </c>
-      <c r="H11" s="58" t="s">
+      <c r="H11" s="47" t="s">
         <v>69</v>
       </c>
-      <c r="I11" s="58"/>
-      <c r="J11" s="58" t="s">
+      <c r="I11" s="47"/>
+      <c r="J11" s="47" t="s">
         <v>66</v>
       </c>
-      <c r="K11" s="58"/>
-      <c r="L11" s="58" t="s">
+      <c r="K11" s="47"/>
+      <c r="L11" s="47" t="s">
         <v>37</v>
       </c>
       <c r="M11" s="24" t="s">
@@ -2908,132 +3064,173 @@
       <c r="A12" s="25" t="s">
         <v>31</v>
       </c>
-      <c r="B12" s="60"/>
-      <c r="C12" s="60"/>
-      <c r="D12" s="60"/>
-      <c r="E12" s="60"/>
-      <c r="F12" s="60"/>
-      <c r="G12" s="60"/>
-      <c r="H12" s="60"/>
-      <c r="I12" s="60"/>
-      <c r="J12" s="60"/>
-      <c r="K12" s="60"/>
-      <c r="L12" s="60"/>
+      <c r="B12" s="49"/>
+      <c r="C12" s="49"/>
+      <c r="D12" s="49"/>
+      <c r="E12" s="49"/>
+      <c r="F12" s="49"/>
+      <c r="G12" s="49"/>
+      <c r="H12" s="49"/>
+      <c r="I12" s="49"/>
+      <c r="J12" s="49"/>
+      <c r="K12" s="49"/>
+      <c r="L12" s="49"/>
       <c r="M12" s="32" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="13" spans="1:14" ht="86.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="103" t="s">
+      <c r="A13" s="74" t="s">
         <v>31</v>
       </c>
-      <c r="B13" s="58" t="s">
+      <c r="B13" s="47" t="s">
         <v>92</v>
       </c>
-      <c r="C13" s="58" t="s">
+      <c r="C13" s="47" t="s">
         <v>93</v>
       </c>
-      <c r="D13" s="58" t="s">
+      <c r="D13" s="47" t="s">
         <v>94</v>
       </c>
-      <c r="E13" s="58" t="s">
+      <c r="E13" s="47" t="s">
         <v>63</v>
       </c>
-      <c r="F13" s="58" t="s">
+      <c r="F13" s="47" t="s">
         <v>95</v>
       </c>
-      <c r="G13" s="43" t="s">
+      <c r="G13" s="44" t="s">
         <v>75</v>
       </c>
-      <c r="H13" s="43" t="s">
+      <c r="H13" s="44" t="s">
         <v>96</v>
       </c>
-      <c r="I13" s="58"/>
-      <c r="J13" s="58" t="s">
+      <c r="I13" s="47"/>
+      <c r="J13" s="47" t="s">
         <v>91</v>
       </c>
-      <c r="K13" s="58"/>
-      <c r="L13" s="58" t="s">
+      <c r="K13" s="47"/>
+      <c r="L13" s="47" t="s">
         <v>37</v>
       </c>
-      <c r="M13" s="58" t="s">
+      <c r="M13" s="47" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="14" spans="1:14" ht="98.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="104"/>
-      <c r="B14" s="60"/>
-      <c r="C14" s="60"/>
-      <c r="D14" s="60"/>
-      <c r="E14" s="60"/>
-      <c r="F14" s="60"/>
-      <c r="G14" s="45"/>
-      <c r="H14" s="45"/>
-      <c r="I14" s="60"/>
-      <c r="J14" s="60"/>
-      <c r="K14" s="60"/>
-      <c r="L14" s="60"/>
-      <c r="M14" s="60"/>
+      <c r="A14" s="75"/>
+      <c r="B14" s="49"/>
+      <c r="C14" s="49"/>
+      <c r="D14" s="49"/>
+      <c r="E14" s="49"/>
+      <c r="F14" s="49"/>
+      <c r="G14" s="46"/>
+      <c r="H14" s="46"/>
+      <c r="I14" s="49"/>
+      <c r="J14" s="49"/>
+      <c r="K14" s="49"/>
+      <c r="L14" s="49"/>
+      <c r="M14" s="49"/>
     </row>
     <row r="15" spans="1:14" ht="120.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="102" t="s">
+      <c r="A15" s="73" t="s">
         <v>31</v>
       </c>
-      <c r="B15" s="102" t="s">
+      <c r="B15" s="73" t="s">
         <v>176</v>
       </c>
-      <c r="C15" s="102" t="s">
+      <c r="C15" s="73" t="s">
         <v>73</v>
       </c>
-      <c r="D15" s="102" t="s">
+      <c r="D15" s="73" t="s">
         <v>30</v>
       </c>
-      <c r="E15" s="102" t="s">
+      <c r="E15" s="73" t="s">
         <v>63</v>
       </c>
-      <c r="F15" s="102" t="s">
+      <c r="F15" s="73" t="s">
         <v>74</v>
       </c>
-      <c r="G15" s="43" t="s">
+      <c r="G15" s="44" t="s">
         <v>165</v>
       </c>
-      <c r="H15" s="43" t="s">
+      <c r="H15" s="44" t="s">
         <v>76</v>
       </c>
-      <c r="I15" s="102"/>
-      <c r="J15" s="102" t="s">
+      <c r="I15" s="73"/>
+      <c r="J15" s="73" t="s">
         <v>38</v>
       </c>
-      <c r="K15" s="102"/>
-      <c r="L15" s="102" t="s">
+      <c r="K15" s="73"/>
+      <c r="L15" s="73" t="s">
         <v>37</v>
       </c>
-      <c r="M15" s="102" t="s">
+      <c r="M15" s="73" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="16" spans="1:14" ht="62.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="102"/>
-      <c r="B16" s="102"/>
-      <c r="C16" s="102"/>
-      <c r="D16" s="102"/>
-      <c r="E16" s="102"/>
-      <c r="F16" s="102"/>
-      <c r="G16" s="45"/>
-      <c r="H16" s="45"/>
-      <c r="I16" s="102"/>
-      <c r="J16" s="102"/>
-      <c r="K16" s="102"/>
-      <c r="L16" s="102"/>
-      <c r="M16" s="102"/>
+      <c r="A16" s="73"/>
+      <c r="B16" s="73"/>
+      <c r="C16" s="73"/>
+      <c r="D16" s="73"/>
+      <c r="E16" s="73"/>
+      <c r="F16" s="73"/>
+      <c r="G16" s="46"/>
+      <c r="H16" s="46"/>
+      <c r="I16" s="73"/>
+      <c r="J16" s="73"/>
+      <c r="K16" s="73"/>
+      <c r="L16" s="73"/>
+      <c r="M16" s="73"/>
     </row>
   </sheetData>
   <mergeCells count="67">
-    <mergeCell ref="A7:A10"/>
-    <mergeCell ref="F7:F10"/>
-    <mergeCell ref="E7:E10"/>
-    <mergeCell ref="D7:D10"/>
-    <mergeCell ref="C7:C10"/>
+    <mergeCell ref="G13:G14"/>
+    <mergeCell ref="H13:H14"/>
+    <mergeCell ref="G8:G10"/>
+    <mergeCell ref="H8:H10"/>
+    <mergeCell ref="M8:M9"/>
+    <mergeCell ref="K11:K12"/>
+    <mergeCell ref="L11:L12"/>
+    <mergeCell ref="J11:J12"/>
+    <mergeCell ref="L7:L10"/>
+    <mergeCell ref="K7:K10"/>
+    <mergeCell ref="J7:J10"/>
+    <mergeCell ref="A1:N1"/>
+    <mergeCell ref="B2:M2"/>
+    <mergeCell ref="B3:M3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="L4:L6"/>
+    <mergeCell ref="M4:M6"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="K5:K6"/>
+    <mergeCell ref="I5:I6"/>
+    <mergeCell ref="J5:J6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="B7:B10"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="F11:F12"/>
+    <mergeCell ref="H11:H12"/>
+    <mergeCell ref="G11:G12"/>
+    <mergeCell ref="I11:I12"/>
+    <mergeCell ref="I7:I10"/>
+    <mergeCell ref="F15:F16"/>
+    <mergeCell ref="I15:I16"/>
+    <mergeCell ref="J15:J16"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="G15:G16"/>
+    <mergeCell ref="H15:H16"/>
     <mergeCell ref="K15:K16"/>
     <mergeCell ref="L15:L16"/>
     <mergeCell ref="M15:M16"/>
@@ -3050,52 +3247,11 @@
     <mergeCell ref="M13:M14"/>
     <mergeCell ref="D15:D16"/>
     <mergeCell ref="E15:E16"/>
-    <mergeCell ref="F15:F16"/>
-    <mergeCell ref="I15:I16"/>
-    <mergeCell ref="J15:J16"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="C15:C16"/>
-    <mergeCell ref="G15:G16"/>
-    <mergeCell ref="H15:H16"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="F11:F12"/>
-    <mergeCell ref="H11:H12"/>
-    <mergeCell ref="G11:G12"/>
-    <mergeCell ref="I11:I12"/>
-    <mergeCell ref="I7:I10"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="B7:B10"/>
-    <mergeCell ref="A1:N1"/>
-    <mergeCell ref="B2:M2"/>
-    <mergeCell ref="B3:M3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="E4:F4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="L4:L6"/>
-    <mergeCell ref="M4:M6"/>
-    <mergeCell ref="E5:F5"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="K5:K6"/>
-    <mergeCell ref="I5:I6"/>
-    <mergeCell ref="J5:J6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="G13:G14"/>
-    <mergeCell ref="H13:H14"/>
-    <mergeCell ref="G8:G10"/>
-    <mergeCell ref="H8:H10"/>
-    <mergeCell ref="M8:M9"/>
-    <mergeCell ref="K11:K12"/>
-    <mergeCell ref="L11:L12"/>
-    <mergeCell ref="J11:J12"/>
-    <mergeCell ref="L7:L10"/>
-    <mergeCell ref="K7:K10"/>
-    <mergeCell ref="J7:J10"/>
+    <mergeCell ref="A7:A10"/>
+    <mergeCell ref="F7:F10"/>
+    <mergeCell ref="E7:E10"/>
+    <mergeCell ref="D7:D10"/>
+    <mergeCell ref="C7:C10"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <hyperlinks>
@@ -3133,83 +3289,83 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="57" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
-      <c r="G1" s="46"/>
-      <c r="H1" s="46"/>
-      <c r="I1" s="46"/>
-      <c r="J1" s="46"/>
-      <c r="K1" s="46"/>
-      <c r="L1" s="46"/>
-      <c r="M1" s="46"/>
-      <c r="N1" s="46"/>
+      <c r="B1" s="57"/>
+      <c r="C1" s="57"/>
+      <c r="D1" s="57"/>
+      <c r="E1" s="57"/>
+      <c r="F1" s="57"/>
+      <c r="G1" s="57"/>
+      <c r="H1" s="57"/>
+      <c r="I1" s="57"/>
+      <c r="J1" s="57"/>
+      <c r="K1" s="57"/>
+      <c r="L1" s="57"/>
+      <c r="M1" s="57"/>
+      <c r="N1" s="57"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="56" t="s">
+      <c r="B2" s="66" t="s">
         <v>31</v>
       </c>
-      <c r="C2" s="56"/>
-      <c r="D2" s="56"/>
-      <c r="E2" s="56"/>
-      <c r="F2" s="56"/>
-      <c r="G2" s="56"/>
-      <c r="H2" s="56"/>
-      <c r="I2" s="56"/>
-      <c r="J2" s="56"/>
-      <c r="K2" s="56"/>
-      <c r="L2" s="56"/>
-      <c r="M2" s="57"/>
+      <c r="C2" s="66"/>
+      <c r="D2" s="66"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="66"/>
+      <c r="G2" s="66"/>
+      <c r="H2" s="66"/>
+      <c r="I2" s="66"/>
+      <c r="J2" s="66"/>
+      <c r="K2" s="66"/>
+      <c r="L2" s="66"/>
+      <c r="M2" s="67"/>
       <c r="N2" s="3"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="64" t="str">
+      <c r="B3" s="68" t="str">
         <f>'Listado Objetos de Dominio'!$B$6</f>
         <v xml:space="preserve"> Objeto de dominio que representa el Administrador encargado de hacer la creacion o gestión de las zonas comunes y la gestión de residentes y sus respectivas reservas en caso de ser necesario.</v>
       </c>
-      <c r="C3" s="64"/>
-      <c r="D3" s="64"/>
-      <c r="E3" s="64"/>
-      <c r="F3" s="64"/>
-      <c r="G3" s="64"/>
-      <c r="H3" s="64"/>
-      <c r="I3" s="64"/>
-      <c r="J3" s="64"/>
-      <c r="K3" s="64"/>
-      <c r="L3" s="64"/>
-      <c r="M3" s="65"/>
+      <c r="C3" s="68"/>
+      <c r="D3" s="68"/>
+      <c r="E3" s="68"/>
+      <c r="F3" s="68"/>
+      <c r="G3" s="68"/>
+      <c r="H3" s="68"/>
+      <c r="I3" s="68"/>
+      <c r="J3" s="68"/>
+      <c r="K3" s="68"/>
+      <c r="L3" s="68"/>
+      <c r="M3" s="69"/>
       <c r="N3" s="4"/>
     </row>
     <row r="4" spans="1:14" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="48" t="s">
+      <c r="B4" s="53" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="48"/>
+      <c r="C4" s="53"/>
       <c r="D4" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="E4" s="66" t="s">
+      <c r="E4" s="54" t="s">
         <v>19</v>
       </c>
-      <c r="F4" s="66"/>
-      <c r="G4" s="51" t="s">
+      <c r="F4" s="54"/>
+      <c r="G4" s="61" t="s">
         <v>13</v>
       </c>
-      <c r="H4" s="51"/>
+      <c r="H4" s="61"/>
       <c r="I4" s="9" t="s">
         <v>14</v>
       </c>
@@ -3219,52 +3375,52 @@
       <c r="K4" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="L4" s="54" t="s">
+      <c r="L4" s="64" t="s">
         <v>17</v>
       </c>
-      <c r="M4" s="55" t="s">
+      <c r="M4" s="65" t="s">
         <v>18</v>
       </c>
       <c r="N4" s="4"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A5" s="47" t="s">
+      <c r="A5" s="58" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="48" t="s">
+      <c r="B5" s="53" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="48" t="s">
+      <c r="C5" s="53" t="s">
         <v>0</v>
       </c>
-      <c r="D5" s="67" t="s">
+      <c r="D5" s="55" t="s">
         <v>23</v>
       </c>
-      <c r="E5" s="66" t="s">
+      <c r="E5" s="54" t="s">
         <v>20</v>
       </c>
-      <c r="F5" s="66"/>
-      <c r="G5" s="49" t="s">
+      <c r="F5" s="54"/>
+      <c r="G5" s="59" t="s">
         <v>7</v>
       </c>
-      <c r="H5" s="49"/>
-      <c r="I5" s="52" t="s">
+      <c r="H5" s="59"/>
+      <c r="I5" s="62" t="s">
         <v>15</v>
       </c>
-      <c r="J5" s="53" t="s">
+      <c r="J5" s="63" t="s">
         <v>8</v>
       </c>
-      <c r="K5" s="50" t="s">
+      <c r="K5" s="60" t="s">
         <v>10</v>
       </c>
-      <c r="L5" s="54"/>
-      <c r="M5" s="55"/>
+      <c r="L5" s="64"/>
+      <c r="M5" s="65"/>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A6" s="47"/>
-      <c r="B6" s="48"/>
-      <c r="C6" s="48"/>
-      <c r="D6" s="68"/>
+      <c r="A6" s="58"/>
+      <c r="B6" s="53"/>
+      <c r="C6" s="53"/>
+      <c r="D6" s="56"/>
       <c r="E6" s="11" t="s">
         <v>21</v>
       </c>
@@ -3277,29 +3433,29 @@
       <c r="H6" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="I6" s="52"/>
-      <c r="J6" s="53"/>
-      <c r="K6" s="50"/>
-      <c r="L6" s="54"/>
-      <c r="M6" s="55"/>
+      <c r="I6" s="62"/>
+      <c r="J6" s="63"/>
+      <c r="K6" s="60"/>
+      <c r="L6" s="64"/>
+      <c r="M6" s="65"/>
     </row>
     <row r="7" spans="1:14" ht="90" x14ac:dyDescent="0.25">
-      <c r="A7" s="61" t="s">
+      <c r="A7" s="50" t="s">
         <v>45</v>
       </c>
-      <c r="B7" s="58" t="s">
+      <c r="B7" s="47" t="s">
         <v>77</v>
       </c>
-      <c r="C7" s="58" t="s">
+      <c r="C7" s="47" t="s">
         <v>78</v>
       </c>
-      <c r="D7" s="58" t="s">
+      <c r="D7" s="47" t="s">
         <v>31</v>
       </c>
-      <c r="E7" s="58" t="s">
+      <c r="E7" s="47" t="s">
         <v>79</v>
       </c>
-      <c r="F7" s="58" t="s">
+      <c r="F7" s="47" t="s">
         <v>80</v>
       </c>
       <c r="G7" s="34" t="s">
@@ -3308,12 +3464,12 @@
       <c r="H7" s="34" t="s">
         <v>166</v>
       </c>
-      <c r="I7" s="58"/>
-      <c r="J7" s="58" t="s">
+      <c r="I7" s="47"/>
+      <c r="J7" s="47" t="s">
         <v>39</v>
       </c>
-      <c r="K7" s="58"/>
-      <c r="L7" s="58" t="s">
+      <c r="K7" s="47"/>
+      <c r="L7" s="47" t="s">
         <v>41</v>
       </c>
       <c r="M7" s="26" t="s">
@@ -3321,71 +3477,71 @@
       </c>
     </row>
     <row r="8" spans="1:14" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="62"/>
-      <c r="B8" s="59"/>
-      <c r="C8" s="59"/>
-      <c r="D8" s="59"/>
-      <c r="E8" s="59"/>
-      <c r="F8" s="59"/>
-      <c r="G8" s="43" t="s">
+      <c r="A8" s="51"/>
+      <c r="B8" s="48"/>
+      <c r="C8" s="48"/>
+      <c r="D8" s="48"/>
+      <c r="E8" s="48"/>
+      <c r="F8" s="48"/>
+      <c r="G8" s="44" t="s">
         <v>170</v>
       </c>
-      <c r="H8" s="43" t="s">
+      <c r="H8" s="44" t="s">
         <v>167</v>
       </c>
-      <c r="I8" s="59"/>
-      <c r="J8" s="59"/>
-      <c r="K8" s="59"/>
-      <c r="L8" s="59"/>
+      <c r="I8" s="48"/>
+      <c r="J8" s="48"/>
+      <c r="K8" s="48"/>
+      <c r="L8" s="48"/>
       <c r="M8" s="26" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A9" s="62"/>
-      <c r="B9" s="59"/>
-      <c r="C9" s="59"/>
-      <c r="D9" s="59"/>
-      <c r="E9" s="59"/>
-      <c r="F9" s="59"/>
-      <c r="G9" s="44"/>
-      <c r="H9" s="44"/>
-      <c r="I9" s="59"/>
-      <c r="J9" s="59"/>
-      <c r="K9" s="59"/>
-      <c r="L9" s="59"/>
+      <c r="A9" s="51"/>
+      <c r="B9" s="48"/>
+      <c r="C9" s="48"/>
+      <c r="D9" s="48"/>
+      <c r="E9" s="48"/>
+      <c r="F9" s="48"/>
+      <c r="G9" s="45"/>
+      <c r="H9" s="45"/>
+      <c r="I9" s="48"/>
+      <c r="J9" s="48"/>
+      <c r="K9" s="48"/>
+      <c r="L9" s="48"/>
       <c r="M9" s="108" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A10" s="62"/>
-      <c r="B10" s="59"/>
-      <c r="C10" s="59"/>
-      <c r="D10" s="59"/>
-      <c r="E10" s="59"/>
-      <c r="F10" s="59"/>
-      <c r="G10" s="44"/>
-      <c r="H10" s="44"/>
-      <c r="I10" s="59"/>
-      <c r="J10" s="59"/>
-      <c r="K10" s="59"/>
-      <c r="L10" s="59"/>
+      <c r="A10" s="51"/>
+      <c r="B10" s="48"/>
+      <c r="C10" s="48"/>
+      <c r="D10" s="48"/>
+      <c r="E10" s="48"/>
+      <c r="F10" s="48"/>
+      <c r="G10" s="45"/>
+      <c r="H10" s="45"/>
+      <c r="I10" s="48"/>
+      <c r="J10" s="48"/>
+      <c r="K10" s="48"/>
+      <c r="L10" s="48"/>
       <c r="M10" s="109"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A11" s="63"/>
-      <c r="B11" s="60"/>
-      <c r="C11" s="60"/>
-      <c r="D11" s="60"/>
-      <c r="E11" s="60"/>
-      <c r="F11" s="60"/>
-      <c r="G11" s="45"/>
-      <c r="H11" s="45"/>
-      <c r="I11" s="60"/>
-      <c r="J11" s="60"/>
-      <c r="K11" s="60"/>
-      <c r="L11" s="60"/>
+      <c r="A11" s="52"/>
+      <c r="B11" s="49"/>
+      <c r="C11" s="49"/>
+      <c r="D11" s="49"/>
+      <c r="E11" s="49"/>
+      <c r="F11" s="49"/>
+      <c r="G11" s="46"/>
+      <c r="H11" s="46"/>
+      <c r="I11" s="49"/>
+      <c r="J11" s="49"/>
+      <c r="K11" s="49"/>
+      <c r="L11" s="49"/>
       <c r="M11" s="110"/>
     </row>
     <row r="12" spans="1:14" ht="90" x14ac:dyDescent="0.25">
@@ -3429,33 +3585,33 @@
       <c r="A13" s="25" t="s">
         <v>31</v>
       </c>
-      <c r="B13" s="58" t="s">
+      <c r="B13" s="47" t="s">
         <v>85</v>
       </c>
-      <c r="C13" s="58" t="s">
+      <c r="C13" s="47" t="s">
         <v>86</v>
       </c>
-      <c r="D13" s="58" t="s">
+      <c r="D13" s="47" t="s">
         <v>31</v>
       </c>
-      <c r="E13" s="58" t="s">
+      <c r="E13" s="47" t="s">
         <v>79</v>
       </c>
-      <c r="F13" s="58" t="s">
+      <c r="F13" s="47" t="s">
         <v>88</v>
       </c>
-      <c r="G13" s="102" t="s">
+      <c r="G13" s="73" t="s">
         <v>172</v>
       </c>
-      <c r="H13" s="102" t="s">
-        <v>189</v>
-      </c>
-      <c r="I13" s="58"/>
-      <c r="J13" s="58" t="s">
+      <c r="H13" s="73" t="s">
+        <v>188</v>
+      </c>
+      <c r="I13" s="47"/>
+      <c r="J13" s="47" t="s">
         <v>40</v>
       </c>
-      <c r="K13" s="58"/>
-      <c r="L13" s="58" t="s">
+      <c r="K13" s="47"/>
+      <c r="L13" s="47" t="s">
         <v>104</v>
       </c>
       <c r="M13" s="26" t="s">
@@ -3466,17 +3622,17 @@
       <c r="A14" s="27" t="s">
         <v>43</v>
       </c>
-      <c r="B14" s="60"/>
-      <c r="C14" s="60"/>
-      <c r="D14" s="60"/>
-      <c r="E14" s="60"/>
-      <c r="F14" s="60"/>
-      <c r="G14" s="102"/>
-      <c r="H14" s="102"/>
-      <c r="I14" s="60"/>
-      <c r="J14" s="60"/>
-      <c r="K14" s="60"/>
-      <c r="L14" s="60"/>
+      <c r="B14" s="49"/>
+      <c r="C14" s="49"/>
+      <c r="D14" s="49"/>
+      <c r="E14" s="49"/>
+      <c r="F14" s="49"/>
+      <c r="G14" s="73"/>
+      <c r="H14" s="73"/>
+      <c r="I14" s="49"/>
+      <c r="J14" s="49"/>
+      <c r="K14" s="49"/>
+      <c r="L14" s="49"/>
       <c r="M14" s="30" t="s">
         <v>89</v>
       </c>
@@ -3523,31 +3679,6 @@
     </row>
   </sheetData>
   <mergeCells count="41">
-    <mergeCell ref="A7:A11"/>
-    <mergeCell ref="F7:F11"/>
-    <mergeCell ref="E7:E11"/>
-    <mergeCell ref="D7:D11"/>
-    <mergeCell ref="C7:C11"/>
-    <mergeCell ref="B7:B11"/>
-    <mergeCell ref="K13:K14"/>
-    <mergeCell ref="L13:L14"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="J13:J14"/>
-    <mergeCell ref="G13:G14"/>
-    <mergeCell ref="H13:H14"/>
-    <mergeCell ref="I13:I14"/>
-    <mergeCell ref="K5:K6"/>
-    <mergeCell ref="L7:L11"/>
-    <mergeCell ref="K7:K11"/>
-    <mergeCell ref="J7:J11"/>
-    <mergeCell ref="I7:I11"/>
-    <mergeCell ref="G8:G11"/>
-    <mergeCell ref="H8:H11"/>
-    <mergeCell ref="B13:B14"/>
-    <mergeCell ref="C13:C14"/>
-    <mergeCell ref="D13:D14"/>
-    <mergeCell ref="E13:E14"/>
-    <mergeCell ref="F13:F14"/>
     <mergeCell ref="M9:M11"/>
     <mergeCell ref="D5:D6"/>
     <mergeCell ref="A1:N1"/>
@@ -3564,6 +3695,31 @@
     <mergeCell ref="L4:L6"/>
     <mergeCell ref="M4:M6"/>
     <mergeCell ref="E5:F5"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="D13:D14"/>
+    <mergeCell ref="E13:E14"/>
+    <mergeCell ref="F13:F14"/>
+    <mergeCell ref="K13:K14"/>
+    <mergeCell ref="L13:L14"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="J13:J14"/>
+    <mergeCell ref="G13:G14"/>
+    <mergeCell ref="H13:H14"/>
+    <mergeCell ref="I13:I14"/>
+    <mergeCell ref="K5:K6"/>
+    <mergeCell ref="L7:L11"/>
+    <mergeCell ref="K7:K11"/>
+    <mergeCell ref="J7:J11"/>
+    <mergeCell ref="I7:I11"/>
+    <mergeCell ref="G8:G11"/>
+    <mergeCell ref="H8:H11"/>
+    <mergeCell ref="A7:A11"/>
+    <mergeCell ref="F7:F11"/>
+    <mergeCell ref="E7:E11"/>
+    <mergeCell ref="D7:D11"/>
+    <mergeCell ref="C7:C11"/>
+    <mergeCell ref="B7:B11"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <hyperlinks>
@@ -3604,84 +3760,84 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="57" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
-      <c r="G1" s="46"/>
-      <c r="H1" s="46"/>
-      <c r="I1" s="46"/>
-      <c r="J1" s="46"/>
-      <c r="K1" s="46"/>
-      <c r="L1" s="46"/>
-      <c r="M1" s="46"/>
-      <c r="N1" s="46"/>
+      <c r="B1" s="57"/>
+      <c r="C1" s="57"/>
+      <c r="D1" s="57"/>
+      <c r="E1" s="57"/>
+      <c r="F1" s="57"/>
+      <c r="G1" s="57"/>
+      <c r="H1" s="57"/>
+      <c r="I1" s="57"/>
+      <c r="J1" s="57"/>
+      <c r="K1" s="57"/>
+      <c r="L1" s="57"/>
+      <c r="M1" s="57"/>
+      <c r="N1" s="57"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="72" t="str">
+      <c r="B2" s="78" t="str">
         <f>'Listado Objetos de Dominio'!A7</f>
         <v>ZonaInmueble</v>
       </c>
-      <c r="C2" s="73"/>
-      <c r="D2" s="73"/>
-      <c r="E2" s="73"/>
-      <c r="F2" s="73"/>
-      <c r="G2" s="73"/>
-      <c r="H2" s="73"/>
-      <c r="I2" s="73"/>
-      <c r="J2" s="73"/>
-      <c r="K2" s="73"/>
-      <c r="L2" s="73"/>
-      <c r="M2" s="74"/>
+      <c r="C2" s="79"/>
+      <c r="D2" s="79"/>
+      <c r="E2" s="79"/>
+      <c r="F2" s="79"/>
+      <c r="G2" s="79"/>
+      <c r="H2" s="79"/>
+      <c r="I2" s="79"/>
+      <c r="J2" s="79"/>
+      <c r="K2" s="79"/>
+      <c r="L2" s="79"/>
+      <c r="M2" s="80"/>
       <c r="N2" s="3"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="75" t="str">
+      <c r="B3" s="81" t="str">
         <f>'Listado Objetos de Dominio'!B7</f>
         <v>Objeto de dominio que representa una Zona de Inmuebles en un conjunto residencial se refiere a una agrupación de unidades habitacionales (como una torre, bloque, o lote) que comparten una ubicación física y características comunes dentro del conjunto.</v>
       </c>
-      <c r="C3" s="76"/>
-      <c r="D3" s="76"/>
-      <c r="E3" s="76"/>
-      <c r="F3" s="76"/>
-      <c r="G3" s="76"/>
-      <c r="H3" s="76"/>
-      <c r="I3" s="76"/>
-      <c r="J3" s="76"/>
-      <c r="K3" s="76"/>
-      <c r="L3" s="76"/>
-      <c r="M3" s="77"/>
+      <c r="C3" s="82"/>
+      <c r="D3" s="82"/>
+      <c r="E3" s="82"/>
+      <c r="F3" s="82"/>
+      <c r="G3" s="82"/>
+      <c r="H3" s="82"/>
+      <c r="I3" s="82"/>
+      <c r="J3" s="82"/>
+      <c r="K3" s="82"/>
+      <c r="L3" s="82"/>
+      <c r="M3" s="83"/>
       <c r="N3" s="4"/>
     </row>
     <row r="4" spans="1:14" ht="37.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="78" t="s">
+      <c r="B4" s="84" t="s">
         <v>132</v>
       </c>
-      <c r="C4" s="79"/>
+      <c r="C4" s="85"/>
       <c r="D4" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="E4" s="80" t="s">
+      <c r="E4" s="86" t="s">
         <v>19</v>
       </c>
-      <c r="F4" s="81"/>
-      <c r="G4" s="82" t="s">
+      <c r="F4" s="87"/>
+      <c r="G4" s="88" t="s">
         <v>13</v>
       </c>
-      <c r="H4" s="83"/>
+      <c r="H4" s="89"/>
       <c r="I4" s="9" t="s">
         <v>14</v>
       </c>
@@ -3691,52 +3847,52 @@
       <c r="K4" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="L4" s="84" t="s">
+      <c r="L4" s="90" t="s">
         <v>17</v>
       </c>
-      <c r="M4" s="87" t="s">
+      <c r="M4" s="93" t="s">
         <v>133</v>
       </c>
       <c r="N4" s="4"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A5" s="98" t="s">
+      <c r="A5" s="104" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="100" t="s">
+      <c r="B5" s="76" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="100" t="s">
+      <c r="C5" s="76" t="s">
         <v>0</v>
       </c>
-      <c r="D5" s="67" t="s">
+      <c r="D5" s="55" t="s">
         <v>23</v>
       </c>
-      <c r="E5" s="80" t="s">
+      <c r="E5" s="86" t="s">
         <v>20</v>
       </c>
-      <c r="F5" s="81"/>
-      <c r="G5" s="90" t="s">
+      <c r="F5" s="87"/>
+      <c r="G5" s="96" t="s">
         <v>7</v>
       </c>
-      <c r="H5" s="91"/>
-      <c r="I5" s="94" t="s">
+      <c r="H5" s="97"/>
+      <c r="I5" s="100" t="s">
         <v>15</v>
       </c>
-      <c r="J5" s="96" t="s">
+      <c r="J5" s="102" t="s">
         <v>8</v>
       </c>
-      <c r="K5" s="92" t="s">
+      <c r="K5" s="98" t="s">
         <v>10</v>
       </c>
-      <c r="L5" s="85"/>
-      <c r="M5" s="88"/>
+      <c r="L5" s="91"/>
+      <c r="M5" s="94"/>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A6" s="99"/>
-      <c r="B6" s="101"/>
-      <c r="C6" s="101"/>
-      <c r="D6" s="68"/>
+      <c r="A6" s="105"/>
+      <c r="B6" s="77"/>
+      <c r="C6" s="77"/>
+      <c r="D6" s="56"/>
       <c r="E6" s="11" t="s">
         <v>21</v>
       </c>
@@ -3749,43 +3905,43 @@
       <c r="H6" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="I6" s="95"/>
-      <c r="J6" s="97"/>
-      <c r="K6" s="93"/>
-      <c r="L6" s="86"/>
-      <c r="M6" s="89"/>
+      <c r="I6" s="101"/>
+      <c r="J6" s="103"/>
+      <c r="K6" s="99"/>
+      <c r="L6" s="92"/>
+      <c r="M6" s="95"/>
     </row>
     <row r="7" spans="1:14" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="102" t="s">
+      <c r="A7" s="73" t="s">
         <v>31</v>
       </c>
-      <c r="B7" s="102" t="s">
+      <c r="B7" s="73" t="s">
         <v>174</v>
       </c>
-      <c r="C7" s="102" t="s">
+      <c r="C7" s="73" t="s">
         <v>114</v>
       </c>
-      <c r="D7" s="102" t="s">
+      <c r="D7" s="73" t="s">
         <v>108</v>
       </c>
-      <c r="E7" s="102" t="s">
+      <c r="E7" s="73" t="s">
         <v>63</v>
       </c>
-      <c r="F7" s="102" t="s">
+      <c r="F7" s="73" t="s">
         <v>115</v>
       </c>
-      <c r="G7" s="102" t="s">
+      <c r="G7" s="73" t="s">
         <v>134</v>
       </c>
-      <c r="H7" s="102" t="s">
-        <v>188</v>
-      </c>
-      <c r="I7" s="102"/>
-      <c r="J7" s="102" t="s">
+      <c r="H7" s="73" t="s">
+        <v>187</v>
+      </c>
+      <c r="I7" s="73"/>
+      <c r="J7" s="73" t="s">
         <v>116</v>
       </c>
-      <c r="K7" s="102"/>
-      <c r="L7" s="102" t="s">
+      <c r="K7" s="73"/>
+      <c r="L7" s="73" t="s">
         <v>117</v>
       </c>
       <c r="M7" s="22" t="s">
@@ -3793,35 +3949,35 @@
       </c>
     </row>
     <row r="8" spans="1:14" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="102"/>
-      <c r="B8" s="102"/>
-      <c r="C8" s="102"/>
-      <c r="D8" s="102"/>
-      <c r="E8" s="102"/>
-      <c r="F8" s="102"/>
-      <c r="G8" s="102"/>
-      <c r="H8" s="102"/>
-      <c r="I8" s="102"/>
-      <c r="J8" s="102"/>
-      <c r="K8" s="102"/>
-      <c r="L8" s="102"/>
+      <c r="A8" s="73"/>
+      <c r="B8" s="73"/>
+      <c r="C8" s="73"/>
+      <c r="D8" s="73"/>
+      <c r="E8" s="73"/>
+      <c r="F8" s="73"/>
+      <c r="G8" s="73"/>
+      <c r="H8" s="73"/>
+      <c r="I8" s="73"/>
+      <c r="J8" s="73"/>
+      <c r="K8" s="73"/>
+      <c r="L8" s="73"/>
       <c r="M8" s="22" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="9" spans="1:14" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="102"/>
-      <c r="B9" s="102"/>
-      <c r="C9" s="102"/>
-      <c r="D9" s="102"/>
-      <c r="E9" s="102"/>
-      <c r="F9" s="102"/>
-      <c r="G9" s="102"/>
-      <c r="H9" s="102"/>
-      <c r="I9" s="102"/>
-      <c r="J9" s="102"/>
-      <c r="K9" s="102"/>
-      <c r="L9" s="102"/>
+      <c r="A9" s="73"/>
+      <c r="B9" s="73"/>
+      <c r="C9" s="73"/>
+      <c r="D9" s="73"/>
+      <c r="E9" s="73"/>
+      <c r="F9" s="73"/>
+      <c r="G9" s="73"/>
+      <c r="H9" s="73"/>
+      <c r="I9" s="73"/>
+      <c r="J9" s="73"/>
+      <c r="K9" s="73"/>
+      <c r="L9" s="73"/>
       <c r="M9" s="22" t="s">
         <v>120</v>
       </c>
@@ -3830,33 +3986,33 @@
       <c r="A10" s="22" t="s">
         <v>43</v>
       </c>
-      <c r="B10" s="102" t="s">
+      <c r="B10" s="73" t="s">
         <v>121</v>
       </c>
-      <c r="C10" s="102" t="s">
+      <c r="C10" s="73" t="s">
         <v>122</v>
       </c>
-      <c r="D10" s="102" t="s">
+      <c r="D10" s="73" t="s">
         <v>108</v>
       </c>
-      <c r="E10" s="102" t="s">
+      <c r="E10" s="73" t="s">
         <v>63</v>
       </c>
-      <c r="F10" s="102" t="s">
+      <c r="F10" s="73" t="s">
         <v>123</v>
       </c>
-      <c r="G10" s="102" t="s">
+      <c r="G10" s="73" t="s">
         <v>178</v>
       </c>
-      <c r="H10" s="102" t="s">
-        <v>183</v>
-      </c>
-      <c r="I10" s="102"/>
-      <c r="J10" s="102" t="s">
+      <c r="H10" s="73" t="s">
+        <v>182</v>
+      </c>
+      <c r="I10" s="73"/>
+      <c r="J10" s="73" t="s">
         <v>124</v>
       </c>
-      <c r="K10" s="102"/>
-      <c r="L10" s="102" t="s">
+      <c r="K10" s="73"/>
+      <c r="L10" s="73" t="s">
         <v>116</v>
       </c>
       <c r="M10" s="22" t="s">
@@ -3867,17 +4023,17 @@
       <c r="A11" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="B11" s="102"/>
-      <c r="C11" s="102"/>
-      <c r="D11" s="102"/>
-      <c r="E11" s="102"/>
-      <c r="F11" s="102"/>
-      <c r="G11" s="102"/>
-      <c r="H11" s="102"/>
-      <c r="I11" s="102"/>
-      <c r="J11" s="102"/>
-      <c r="K11" s="102"/>
-      <c r="L11" s="102"/>
+      <c r="B11" s="73"/>
+      <c r="C11" s="73"/>
+      <c r="D11" s="73"/>
+      <c r="E11" s="73"/>
+      <c r="F11" s="73"/>
+      <c r="G11" s="73"/>
+      <c r="H11" s="73"/>
+      <c r="I11" s="73"/>
+      <c r="J11" s="73"/>
+      <c r="K11" s="73"/>
+      <c r="L11" s="73"/>
       <c r="M11" s="22" t="s">
         <v>120</v>
       </c>
@@ -3958,30 +4114,6 @@
     </row>
   </sheetData>
   <mergeCells count="40">
-    <mergeCell ref="A1:N1"/>
-    <mergeCell ref="B2:M2"/>
-    <mergeCell ref="B3:M3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="E4:F4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="L4:L6"/>
-    <mergeCell ref="M4:M6"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="K5:K6"/>
-    <mergeCell ref="A7:A9"/>
-    <mergeCell ref="B7:B9"/>
-    <mergeCell ref="C7:C9"/>
-    <mergeCell ref="D7:D9"/>
-    <mergeCell ref="E7:E9"/>
-    <mergeCell ref="J7:J9"/>
-    <mergeCell ref="K7:K9"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:F5"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="I5:I6"/>
-    <mergeCell ref="J5:J6"/>
     <mergeCell ref="L10:L11"/>
     <mergeCell ref="L7:L9"/>
     <mergeCell ref="B10:B11"/>
@@ -3998,6 +4130,30 @@
     <mergeCell ref="K10:K11"/>
     <mergeCell ref="F7:F9"/>
     <mergeCell ref="I7:I9"/>
+    <mergeCell ref="J7:J9"/>
+    <mergeCell ref="K7:K9"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="I5:I6"/>
+    <mergeCell ref="J5:J6"/>
+    <mergeCell ref="A7:A9"/>
+    <mergeCell ref="B7:B9"/>
+    <mergeCell ref="C7:C9"/>
+    <mergeCell ref="D7:D9"/>
+    <mergeCell ref="E7:E9"/>
+    <mergeCell ref="A1:N1"/>
+    <mergeCell ref="B2:M2"/>
+    <mergeCell ref="B3:M3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="L4:L6"/>
+    <mergeCell ref="M4:M6"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="K5:K6"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A1" location="'Objetos de Dominio'!A1" display="Volver al inicio" xr:uid="{40DB47AD-DF64-4401-B17F-CC72FC22A8C4}"/>
@@ -4009,7 +4165,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25B1D8D7-0621-4D6B-8ACC-3788EF366C74}">
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -4035,360 +4191,449 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="57" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
-      <c r="G1" s="46"/>
-      <c r="H1" s="46"/>
-      <c r="I1" s="46"/>
-      <c r="J1" s="46"/>
-      <c r="K1" s="46"/>
-      <c r="L1" s="46"/>
-      <c r="M1" s="46"/>
-      <c r="N1" s="46"/>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
+      <c r="B1" s="57"/>
+      <c r="C1" s="57"/>
+      <c r="D1" s="57"/>
+      <c r="E1" s="57"/>
+      <c r="F1" s="57"/>
+      <c r="G1" s="57"/>
+      <c r="H1" s="57"/>
+      <c r="I1" s="57"/>
+      <c r="J1" s="57"/>
+      <c r="K1" s="57"/>
+      <c r="L1" s="57"/>
+      <c r="M1" s="57"/>
+      <c r="N1" s="57"/>
+    </row>
+    <row r="2" spans="1:14" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="111" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="72" t="str">
-        <f>'Listado Objetos de Dominio'!A7</f>
-        <v>ZonaInmueble</v>
-      </c>
-      <c r="C2" s="73"/>
-      <c r="D2" s="73"/>
-      <c r="E2" s="73"/>
-      <c r="F2" s="73"/>
-      <c r="G2" s="73"/>
-      <c r="H2" s="73"/>
-      <c r="I2" s="73"/>
-      <c r="J2" s="73"/>
-      <c r="K2" s="73"/>
-      <c r="L2" s="73"/>
-      <c r="M2" s="74"/>
+      <c r="B2" s="112" t="str">
+        <f>'Listado Objetos de Dominio'!A8</f>
+        <v>Inmueble</v>
+      </c>
+      <c r="C2" s="112"/>
+      <c r="D2" s="112"/>
+      <c r="E2" s="112"/>
+      <c r="F2" s="112"/>
+      <c r="G2" s="112"/>
+      <c r="H2" s="112"/>
+      <c r="I2" s="112"/>
+      <c r="J2" s="112"/>
+      <c r="K2" s="112"/>
+      <c r="L2" s="112"/>
+      <c r="M2" s="112"/>
       <c r="N2" s="3"/>
     </row>
-    <row r="3" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
+    <row r="3" spans="1:14" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="111" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="75" t="str">
-        <f>'Listado Objetos de Dominio'!B7</f>
-        <v>Objeto de dominio que representa una Zona de Inmuebles en un conjunto residencial se refiere a una agrupación de unidades habitacionales (como una torre, bloque, o lote) que comparten una ubicación física y características comunes dentro del conjunto.</v>
-      </c>
-      <c r="C3" s="76"/>
-      <c r="D3" s="76"/>
-      <c r="E3" s="76"/>
-      <c r="F3" s="76"/>
-      <c r="G3" s="76"/>
-      <c r="H3" s="76"/>
-      <c r="I3" s="76"/>
-      <c r="J3" s="76"/>
-      <c r="K3" s="76"/>
-      <c r="L3" s="76"/>
-      <c r="M3" s="77"/>
+      <c r="B3" s="113" t="str">
+        <f>'Listado Objetos de Dominio'!B8</f>
+        <v>Objeto de dominio que representa un inmueble dentro de una zona de inmuebles en un conjunto residencial describe las características específicas de una unidad habitacional en el contexto de una agrupación más amplia, como una torre, bloque o área específica, que es representada por su zona de inmueble</v>
+      </c>
+      <c r="C3" s="113"/>
+      <c r="D3" s="113"/>
+      <c r="E3" s="113"/>
+      <c r="F3" s="113"/>
+      <c r="G3" s="113"/>
+      <c r="H3" s="113"/>
+      <c r="I3" s="113"/>
+      <c r="J3" s="113"/>
+      <c r="K3" s="113"/>
+      <c r="L3" s="113"/>
+      <c r="M3" s="113"/>
       <c r="N3" s="4"/>
     </row>
-    <row r="4" spans="1:14" ht="37.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="8" t="s">
+    <row r="4" spans="1:14" ht="37.15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="114" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="78" t="s">
+      <c r="B4" s="115" t="s">
         <v>132</v>
       </c>
-      <c r="C4" s="79"/>
-      <c r="D4" s="13" t="s">
+      <c r="C4" s="115"/>
+      <c r="D4" s="116" t="s">
         <v>22</v>
       </c>
-      <c r="E4" s="80" t="s">
+      <c r="E4" s="117" t="s">
         <v>19</v>
       </c>
-      <c r="F4" s="81"/>
-      <c r="G4" s="82" t="s">
+      <c r="F4" s="117"/>
+      <c r="G4" s="118" t="s">
         <v>13</v>
       </c>
-      <c r="H4" s="83"/>
-      <c r="I4" s="9" t="s">
+      <c r="H4" s="118"/>
+      <c r="I4" s="119" t="s">
         <v>14</v>
       </c>
-      <c r="J4" s="10" t="s">
+      <c r="J4" s="120" t="s">
         <v>11</v>
       </c>
-      <c r="K4" s="12" t="s">
+      <c r="K4" s="121" t="s">
         <v>16</v>
       </c>
-      <c r="L4" s="84" t="s">
+      <c r="L4" s="122" t="s">
         <v>17</v>
       </c>
-      <c r="M4" s="87" t="s">
+      <c r="M4" s="123" t="s">
         <v>133</v>
       </c>
       <c r="N4" s="4"/>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A5" s="98" t="s">
+    <row r="5" spans="1:14" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="124" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="100" t="s">
+      <c r="B5" s="115" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="100" t="s">
+      <c r="C5" s="115" t="s">
         <v>0</v>
       </c>
-      <c r="D5" s="67" t="s">
+      <c r="D5" s="125" t="s">
         <v>23</v>
       </c>
-      <c r="E5" s="80" t="s">
+      <c r="E5" s="117" t="s">
         <v>20</v>
       </c>
-      <c r="F5" s="81"/>
-      <c r="G5" s="90" t="s">
+      <c r="F5" s="117"/>
+      <c r="G5" s="126" t="s">
         <v>7</v>
       </c>
-      <c r="H5" s="91"/>
-      <c r="I5" s="94" t="s">
+      <c r="H5" s="126"/>
+      <c r="I5" s="127" t="s">
         <v>15</v>
       </c>
-      <c r="J5" s="96" t="s">
+      <c r="J5" s="128" t="s">
         <v>8</v>
       </c>
-      <c r="K5" s="92" t="s">
+      <c r="K5" s="129" t="s">
         <v>10</v>
       </c>
-      <c r="L5" s="85"/>
-      <c r="M5" s="88"/>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A6" s="99"/>
-      <c r="B6" s="101"/>
-      <c r="C6" s="101"/>
-      <c r="D6" s="68"/>
-      <c r="E6" s="11" t="s">
+      <c r="L5" s="122"/>
+      <c r="M5" s="123"/>
+    </row>
+    <row r="6" spans="1:14" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="124"/>
+      <c r="B6" s="115"/>
+      <c r="C6" s="115"/>
+      <c r="D6" s="125"/>
+      <c r="E6" s="130" t="s">
         <v>21</v>
       </c>
-      <c r="F6" s="11" t="s">
+      <c r="F6" s="130" t="s">
         <v>0</v>
       </c>
-      <c r="G6" s="7" t="s">
+      <c r="G6" s="131" t="s">
         <v>9</v>
       </c>
-      <c r="H6" s="7" t="s">
+      <c r="H6" s="131" t="s">
         <v>0</v>
       </c>
-      <c r="I6" s="95"/>
-      <c r="J6" s="97"/>
-      <c r="K6" s="93"/>
-      <c r="L6" s="86"/>
-      <c r="M6" s="89"/>
-    </row>
-    <row r="7" spans="1:14" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="102" t="s">
+      <c r="I6" s="127"/>
+      <c r="J6" s="128"/>
+      <c r="K6" s="129"/>
+      <c r="L6" s="122"/>
+      <c r="M6" s="123"/>
+    </row>
+    <row r="7" spans="1:14" ht="106.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="132" t="s">
         <v>31</v>
       </c>
-      <c r="B7" s="102" t="s">
+      <c r="B7" s="132" t="s">
         <v>141</v>
       </c>
-      <c r="C7" s="102" t="s">
+      <c r="C7" s="132" t="s">
         <v>142</v>
       </c>
-      <c r="D7" s="102" t="s">
+      <c r="D7" s="132" t="s">
         <v>109</v>
       </c>
-      <c r="E7" s="102" t="s">
+      <c r="E7" s="132" t="s">
         <v>151</v>
       </c>
-      <c r="F7" s="102" t="s">
+      <c r="F7" s="132" t="s">
         <v>152</v>
       </c>
-      <c r="G7" s="102" t="s">
+      <c r="G7" s="133" t="s">
         <v>157</v>
       </c>
-      <c r="H7" s="102" t="s">
-        <v>187</v>
-      </c>
-      <c r="I7" s="102"/>
-      <c r="J7" s="102" t="s">
+      <c r="H7" s="133" t="s">
+        <v>186</v>
+      </c>
+      <c r="I7" s="132"/>
+      <c r="J7" s="132" t="s">
         <v>136</v>
       </c>
-      <c r="K7" s="102"/>
-      <c r="L7" s="102" t="s">
+      <c r="K7" s="132"/>
+      <c r="L7" s="132" t="s">
         <v>143</v>
       </c>
-      <c r="M7" s="22" t="s">
+      <c r="M7" s="134" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="8" spans="1:14" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="102"/>
-      <c r="B8" s="102"/>
-      <c r="C8" s="102"/>
-      <c r="D8" s="102"/>
-      <c r="E8" s="102"/>
-      <c r="F8" s="102"/>
-      <c r="G8" s="102"/>
-      <c r="H8" s="102"/>
-      <c r="I8" s="102"/>
-      <c r="J8" s="102"/>
-      <c r="K8" s="102"/>
-      <c r="L8" s="102"/>
-      <c r="M8" s="22" t="s">
+    <row r="8" spans="1:14" ht="76.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="132"/>
+      <c r="B8" s="132"/>
+      <c r="C8" s="132"/>
+      <c r="D8" s="132"/>
+      <c r="E8" s="132"/>
+      <c r="F8" s="132"/>
+      <c r="G8" s="133" t="s">
+        <v>183</v>
+      </c>
+      <c r="H8" s="133" t="s">
+        <v>194</v>
+      </c>
+      <c r="I8" s="132"/>
+      <c r="J8" s="132"/>
+      <c r="K8" s="132"/>
+      <c r="L8" s="132"/>
+      <c r="M8" s="134" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="102"/>
-      <c r="B9" s="102"/>
-      <c r="C9" s="102"/>
-      <c r="D9" s="102"/>
-      <c r="E9" s="102"/>
-      <c r="F9" s="102"/>
-      <c r="G9" s="102"/>
-      <c r="H9" s="102"/>
-      <c r="I9" s="102"/>
-      <c r="J9" s="102"/>
-      <c r="K9" s="102"/>
-      <c r="L9" s="102"/>
-      <c r="M9" s="22" t="s">
+    <row r="9" spans="1:14" ht="46.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="132"/>
+      <c r="B9" s="132"/>
+      <c r="C9" s="132"/>
+      <c r="D9" s="132"/>
+      <c r="E9" s="132"/>
+      <c r="F9" s="132"/>
+      <c r="G9" s="133" t="s">
+        <v>184</v>
+      </c>
+      <c r="H9" s="133" t="s">
+        <v>195</v>
+      </c>
+      <c r="I9" s="132"/>
+      <c r="J9" s="132"/>
+      <c r="K9" s="132"/>
+      <c r="L9" s="132"/>
+      <c r="M9" s="134" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="10" spans="1:14" ht="62.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="22" t="s">
-        <v>43</v>
-      </c>
-      <c r="B10" s="102" t="s">
+    <row r="10" spans="1:14" ht="62.45" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="135" t="s">
+        <v>196</v>
+      </c>
+      <c r="B10" s="136" t="s">
         <v>138</v>
       </c>
-      <c r="C10" s="102" t="s">
+      <c r="C10" s="136" t="s">
         <v>147</v>
       </c>
-      <c r="D10" s="102" t="s">
+      <c r="D10" s="136" t="s">
         <v>109</v>
       </c>
-      <c r="E10" s="102" t="s">
+      <c r="E10" s="136" t="s">
         <v>151</v>
       </c>
-      <c r="F10" s="102" t="s">
+      <c r="F10" s="136" t="s">
         <v>153</v>
       </c>
-      <c r="G10" s="102" t="s">
-        <v>184</v>
-      </c>
-      <c r="H10" s="102" t="s">
+      <c r="G10" s="136" t="s">
+        <v>185</v>
+      </c>
+      <c r="H10" s="136" t="s">
+        <v>197</v>
+      </c>
+      <c r="I10" s="136"/>
+      <c r="J10" s="136" t="s">
+        <v>139</v>
+      </c>
+      <c r="K10" s="136"/>
+      <c r="L10" s="137" t="s">
+        <v>135</v>
+      </c>
+      <c r="M10" s="138" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" ht="60.6" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="135" t="s">
+        <v>31</v>
+      </c>
+      <c r="B11" s="136"/>
+      <c r="C11" s="136"/>
+      <c r="D11" s="136"/>
+      <c r="E11" s="136"/>
+      <c r="F11" s="136"/>
+      <c r="G11" s="136"/>
+      <c r="H11" s="136"/>
+      <c r="I11" s="136"/>
+      <c r="J11" s="136"/>
+      <c r="K11" s="136"/>
+      <c r="L11" s="137"/>
+      <c r="M11" s="138" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" ht="105.6" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="139" t="s">
+        <v>31</v>
+      </c>
+      <c r="B12" s="139" t="s">
+        <v>145</v>
+      </c>
+      <c r="C12" s="139" t="s">
+        <v>148</v>
+      </c>
+      <c r="D12" s="139" t="s">
+        <v>150</v>
+      </c>
+      <c r="E12" s="139" t="s">
+        <v>151</v>
+      </c>
+      <c r="F12" s="139" t="s">
+        <v>154</v>
+      </c>
+      <c r="G12" s="140" t="s">
+        <v>198</v>
+      </c>
+      <c r="H12" s="140" t="s">
+        <v>159</v>
+      </c>
+      <c r="I12" s="140"/>
+      <c r="J12" s="139" t="s">
+        <v>137</v>
+      </c>
+      <c r="K12" s="140"/>
+      <c r="L12" s="137"/>
+      <c r="M12" s="137" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" ht="105.6" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="139"/>
+      <c r="B13" s="139"/>
+      <c r="C13" s="139"/>
+      <c r="D13" s="139"/>
+      <c r="E13" s="139"/>
+      <c r="F13" s="139"/>
+      <c r="G13" s="140" t="s">
+        <v>199</v>
+      </c>
+      <c r="H13" s="140" t="s">
+        <v>200</v>
+      </c>
+      <c r="I13" s="140"/>
+      <c r="J13" s="139"/>
+      <c r="K13" s="140"/>
+      <c r="L13" s="137"/>
+      <c r="M13" s="137"/>
+    </row>
+    <row r="14" spans="1:14" ht="120.6" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="141" t="s">
+        <v>31</v>
+      </c>
+      <c r="B14" s="141" t="s">
+        <v>146</v>
+      </c>
+      <c r="C14" s="141" t="s">
+        <v>155</v>
+      </c>
+      <c r="D14" s="141" t="s">
+        <v>109</v>
+      </c>
+      <c r="E14" s="141" t="s">
+        <v>151</v>
+      </c>
+      <c r="F14" s="141" t="s">
+        <v>156</v>
+      </c>
+      <c r="G14" s="142" t="s">
+        <v>201</v>
+      </c>
+      <c r="H14" s="142" t="s">
         <v>182</v>
       </c>
-      <c r="I10" s="102"/>
-      <c r="J10" s="102" t="s">
-        <v>139</v>
-      </c>
-      <c r="K10" s="102"/>
-      <c r="L10" s="102" t="s">
+      <c r="I14" s="142"/>
+      <c r="J14" s="141" t="s">
+        <v>140</v>
+      </c>
+      <c r="K14" s="142"/>
+      <c r="L14" s="141" t="s">
         <v>135</v>
       </c>
-      <c r="M10" s="22" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" ht="60.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="B11" s="102"/>
-      <c r="C11" s="102"/>
-      <c r="D11" s="102"/>
-      <c r="E11" s="102"/>
-      <c r="F11" s="102"/>
-      <c r="G11" s="102"/>
-      <c r="H11" s="102"/>
-      <c r="I11" s="102"/>
-      <c r="J11" s="102"/>
-      <c r="K11" s="102"/>
-      <c r="L11" s="102"/>
-      <c r="M11" s="22" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" ht="105.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="B12" s="22" t="s">
-        <v>145</v>
-      </c>
-      <c r="C12" s="22" t="s">
-        <v>148</v>
-      </c>
-      <c r="D12" s="22" t="s">
-        <v>150</v>
-      </c>
-      <c r="E12" s="22" t="s">
-        <v>151</v>
-      </c>
-      <c r="F12" s="22" t="s">
-        <v>154</v>
-      </c>
-      <c r="G12" s="22" t="s">
-        <v>185</v>
-      </c>
-      <c r="H12" s="22" t="s">
-        <v>159</v>
-      </c>
-      <c r="I12" s="22"/>
-      <c r="J12" s="22" t="s">
-        <v>137</v>
-      </c>
-      <c r="K12" s="22"/>
-      <c r="L12" s="22" t="s">
-        <v>135</v>
-      </c>
-      <c r="M12" s="22" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" ht="120.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="B13" s="22" t="s">
-        <v>146</v>
-      </c>
-      <c r="C13" s="22" t="s">
-        <v>155</v>
-      </c>
-      <c r="D13" s="22" t="s">
-        <v>109</v>
-      </c>
-      <c r="E13" s="22" t="s">
-        <v>151</v>
-      </c>
-      <c r="F13" s="22" t="s">
-        <v>156</v>
-      </c>
-      <c r="G13" s="22" t="s">
-        <v>186</v>
-      </c>
-      <c r="H13" s="22" t="s">
-        <v>183</v>
-      </c>
-      <c r="I13" s="22"/>
-      <c r="J13" s="22" t="s">
-        <v>140</v>
-      </c>
-      <c r="K13" s="22"/>
-      <c r="L13" s="22" t="s">
-        <v>135</v>
-      </c>
-      <c r="M13" s="22" t="s">
+      <c r="M14" s="142" t="s">
         <v>149</v>
       </c>
     </row>
+    <row r="15" spans="1:14" ht="120.6" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="141"/>
+      <c r="B15" s="141"/>
+      <c r="C15" s="141"/>
+      <c r="D15" s="141"/>
+      <c r="E15" s="141"/>
+      <c r="F15" s="141"/>
+      <c r="G15" s="142" t="s">
+        <v>202</v>
+      </c>
+      <c r="H15" s="142" t="s">
+        <v>203</v>
+      </c>
+      <c r="I15" s="142"/>
+      <c r="J15" s="141"/>
+      <c r="K15" s="142"/>
+      <c r="L15" s="141"/>
+      <c r="M15" s="142" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="40">
+  <mergeCells count="54">
+    <mergeCell ref="M12:M13"/>
+    <mergeCell ref="F14:F15"/>
+    <mergeCell ref="L14:L15"/>
+    <mergeCell ref="J14:J15"/>
+    <mergeCell ref="J12:J13"/>
+    <mergeCell ref="L10:L13"/>
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="C14:C15"/>
+    <mergeCell ref="D14:D15"/>
+    <mergeCell ref="E14:E15"/>
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="D12:D13"/>
+    <mergeCell ref="E12:E13"/>
+    <mergeCell ref="F12:F13"/>
+    <mergeCell ref="I10:I11"/>
+    <mergeCell ref="J10:J11"/>
+    <mergeCell ref="K10:K11"/>
+    <mergeCell ref="J7:J9"/>
+    <mergeCell ref="K7:K9"/>
+    <mergeCell ref="L7:L9"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="D10:D11"/>
+    <mergeCell ref="E10:E11"/>
+    <mergeCell ref="F10:F11"/>
+    <mergeCell ref="G10:G11"/>
+    <mergeCell ref="H10:H11"/>
+    <mergeCell ref="K5:K6"/>
+    <mergeCell ref="A7:A9"/>
+    <mergeCell ref="B7:B9"/>
+    <mergeCell ref="C7:C9"/>
+    <mergeCell ref="D7:D9"/>
+    <mergeCell ref="E7:E9"/>
+    <mergeCell ref="F7:F9"/>
+    <mergeCell ref="I7:I9"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="G5:H5"/>
     <mergeCell ref="I5:I6"/>
     <mergeCell ref="J5:J6"/>
     <mergeCell ref="A1:N1"/>
@@ -4401,34 +4646,6 @@
     <mergeCell ref="M4:M6"/>
     <mergeCell ref="A5:A6"/>
     <mergeCell ref="B5:B6"/>
-    <mergeCell ref="G10:G11"/>
-    <mergeCell ref="H10:H11"/>
-    <mergeCell ref="K5:K6"/>
-    <mergeCell ref="A7:A9"/>
-    <mergeCell ref="B7:B9"/>
-    <mergeCell ref="C7:C9"/>
-    <mergeCell ref="D7:D9"/>
-    <mergeCell ref="E7:E9"/>
-    <mergeCell ref="F7:F9"/>
-    <mergeCell ref="G7:G9"/>
-    <mergeCell ref="H7:H9"/>
-    <mergeCell ref="I7:I9"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:F5"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="B10:B11"/>
-    <mergeCell ref="C10:C11"/>
-    <mergeCell ref="D10:D11"/>
-    <mergeCell ref="E10:E11"/>
-    <mergeCell ref="F10:F11"/>
-    <mergeCell ref="I10:I11"/>
-    <mergeCell ref="J10:J11"/>
-    <mergeCell ref="K10:K11"/>
-    <mergeCell ref="L10:L11"/>
-    <mergeCell ref="J7:J9"/>
-    <mergeCell ref="K7:K9"/>
-    <mergeCell ref="L7:L9"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A1" location="'Objetos de Dominio'!A1" display="Volver al inicio" xr:uid="{DE0AC091-170B-4F28-806F-0CE19EF466E0}"/>
@@ -4439,6 +4656,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C279D002CEC08F42B7087C30E58D0266" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e5713f579c7011938dc4987ae8981b8f">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3219184d-29ab-4105-b29c-8e343e335d59" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ae0a0ff84a3c6712467f60982d6e378d" ns2:_="">
     <xsd:import namespace="3219184d-29ab-4105-b29c-8e343e335d59"/>
@@ -4582,35 +4814,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8AEECCE0-61F9-4782-94C5-382F8EFF459D}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6724C681-8A04-4D66-BB1C-57F7466573C0}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="3219184d-29ab-4105-b29c-8e343e335d59"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -4633,9 +4840,19 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6724C681-8A04-4D66-BB1C-57F7466573C0}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8AEECCE0-61F9-4782-94C5-382F8EFF459D}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="3219184d-29ab-4105-b29c-8e343e335d59"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>